<commit_message>
Configure REFramework init, folders, workbook setup, and Groq API handling
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Learning\UiPath\UiPath Tutorial &amp; Projects\Projects\InvoiceProcessor.GenAI\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2CCA52A6-278E-419A-A739-A6107B0016E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55BE0911-B997-4AD6-B881-8C2419DB187D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="6915" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1520" yWindow="1520" windowWidth="19200" windowHeight="10050" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="86">
   <si>
     <t>Name</t>
   </si>
@@ -691,14 +691,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="52" customWidth="1"/>
     <col min="3" max="3" width="62" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -709,7 +709,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="26" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -720,7 +720,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="26" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>6</v>
       </c>
@@ -729,7 +729,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="26" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>8</v>
       </c>
@@ -740,7 +740,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
         <v>11</v>
       </c>
@@ -751,7 +751,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
         <v>14</v>
       </c>
@@ -762,7 +762,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
         <v>17</v>
       </c>
@@ -773,7 +773,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
         <v>20</v>
       </c>
@@ -784,7 +784,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
         <v>23</v>
       </c>
@@ -795,7 +795,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
         <v>26</v>
       </c>
@@ -806,7 +806,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
         <v>29</v>
       </c>
@@ -817,7 +817,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="26" x14ac:dyDescent="0.35">
       <c r="A12" s="6" t="s">
         <v>32</v>
       </c>
@@ -836,14 +836,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
     <col min="2" max="2" width="52" customWidth="1"/>
     <col min="3" max="3" width="62" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -854,7 +854,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="26" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>35</v>
       </c>
@@ -865,7 +865,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>38</v>
       </c>
@@ -876,7 +876,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>41</v>
       </c>
@@ -887,7 +887,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
         <v>44</v>
       </c>
@@ -898,7 +898,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>47</v>
       </c>
@@ -909,7 +909,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>50</v>
       </c>
@@ -920,7 +920,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
         <v>53</v>
       </c>
@@ -931,7 +931,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
         <v>56</v>
       </c>
@@ -942,7 +942,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" ht="26" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
         <v>59</v>
       </c>
@@ -953,7 +953,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
         <v>62</v>
       </c>
@@ -964,7 +964,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
         <v>64</v>
       </c>
@@ -975,7 +975,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="26" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
         <v>66</v>
       </c>
@@ -986,7 +986,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="26" x14ac:dyDescent="0.35">
       <c r="A14" s="6" t="s">
         <v>69</v>
       </c>
@@ -997,7 +997,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="26" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">
         <v>72</v>
       </c>
@@ -1008,7 +1008,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="26" x14ac:dyDescent="0.35">
       <c r="A16" s="6" t="s">
         <v>75</v>
       </c>
@@ -1019,7 +1019,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" ht="26" x14ac:dyDescent="0.35">
       <c r="A17" s="6" t="s">
         <v>78</v>
       </c>
@@ -1038,14 +1038,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="24" customWidth="1"/>
+    <col min="3" max="3" width="67.26953125" customWidth="1"/>
     <col min="4" max="4" width="62" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1059,13 +1059,11 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="39" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>84</v>
-      </c>
+      <c r="B2" s="6"/>
       <c r="C2" s="6"/>
       <c r="D2" s="7" t="s">
         <v>85</v>

</xml_diff>